<commit_message>
Fix: Corregir receptor y direccion de remision E0071 de Galvatek a EQM
</commit_message>
<xml_diff>
--- a/BD_Datos_Generales_Remision.xlsx
+++ b/BD_Datos_Generales_Remision.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Datos_Sistema" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos_Sistema" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2148,12 +2148,12 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Galvatec Industrias</t>
+          <t>EQM</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Prol. Valle Guadiana 919, Parque Industrial II, 35078 Gómez Palacio, Dgo.</t>
+          <t>Calle Inde 714, 35079 Gómez Palacio, Durango</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">

</xml_diff>